<commit_message>
docs(order-management): lock 24.6 scope — 22 deliverable, derived status display, 24.6 owns installment void; 3 BA clarifications + full Order Status sheet applied
</commit_message>
<xml_diff>
--- a/order_management/24.6-order-details/24.6 - Order Details.xlsx
+++ b/order_management/24.6-order-details/24.6 - Order Details.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,12 @@
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -81,8 +85,28 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -104,11 +128,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -157,6 +195,30 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -574,7 +636,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>27 requirement(s) to implement here (filter Build Focus = 'Implement here'). 1 covered elsewhere, 0 out of scope.</t>
+          <t>SCOPE LOCKED at Step-1 gate 2026-07-03. 22 Deliverable / 1 Deferred / 3 Needs clarification (BA) / 1 Covered elsewhere (24.5, live) / 1 Blocked (epic 65). Ship-together release; builds after 24.8.</t>
         </is>
       </c>
     </row>
@@ -584,8 +646,10 @@
           <t>To implement here</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
-        <v>27</v>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1">
@@ -596,13 +660,21 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Story 24.6 asks for a full admin Order Details page: General info, Billing (editable address + additional emails), Line Items (linked product/show, per-item pricing, sub-items under a parent), Fees, Order Totals with payment-plan + next-installment, Send Order Email, Agreement view/download, Sales-Rep/Deal-Owner assignment with HubSpot sync, QuickBooks force sync, HubSpot manual sync, and role-gated actions. The core read model is strongly backed: Order/OrderItem/OrderAgreement/PaymentTransaction/CartPaymentPlan are real models written by the built checkout flows (admin checkout.service.ts + exhibitor cart/payments paths), so the GET details endpoint, totals, fees, line items, next installment, customer linkage, signer info, and permission gating are Deliverable as net-new endpoints on built primitives. Verified caveats: the full billing-address snapshot is written only on the exhibitor self-service path (payments.service.ts), while the admin checkout writes only company name + first/last + email; parent_order_item_id is set only by the exhibitor cart materialization path, not by admin checkout or the exhibitor payments path. Several spec fields used to live only on the Cart (invoice_note, additional_terms, internal_notes) or not exist at all (Payment Memo) — resolved 2026-07-03 when story 24.14 (SBE-1138) merged to dev, adding all four as Order columns with the canonical PATCH write path, so 24.6-c/d/e/f are now display-only Deliverable. The Additional Emails store still does not exist, and the 6-state status taxonomy still does not map to the OrderStatus enum, keeping those Partial. QuickBooks force sync has zero integration code (Blocked), the HubSpot deal-owner auto-update is Blocked (no updateDeal, no order→deal linkage, no hubspot_deal_id on Order), and refund/void execution has no code (Blocked).</t>
+          <t>Gate outcome: GET :id aggregate + PATCH :id (billing/additional_emails, status-gated) + PATCH :id/sales-rep + 24.6-OWNED per-installment void (D-z). Status = derived 6-value display mapping (D1, no migration; qualifiers from 24.9 ledger). Rep/source = read-time derivation (D3/D4, 'Self-Service' default per story). additional_emails = Json column (D5). Admin-checkout snapshot gaps registered to Cart Mgmt team (D2/OQ-1) — page renders gracefully. Parked: send-email (OQ-4), HubSpot v/x (OQ-5 — no owning epic). Deferred: l2 onsite contact (SBE-1169/1171). Blocked: w on QB epic 65. Order Status sheet fetched in full (6 tabs) and applied; label map + edit-rules matrix sourced from it.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Deferred / Parked / Covered / Blocked</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>1 Deferred (l2) · 3 Needs clarification (r, v, x) · 1 Covered by 24.5 (s) · 1 Blocked (w)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -621,23 +693,23 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Needs clarification (BA)</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
@@ -647,21 +719,21 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Not Deliverable</t>
+          <t>Covered elsewhere</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Out of Scope</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -672,7 +744,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Not started — analysis only</t>
+          <t>Not started — scope locked 2026-07-03 (gate complete); plan after full 7-story gate</t>
         </is>
       </c>
     </row>
@@ -798,7 +870,7 @@
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>Impl Status (2026-07-01)</t>
+          <t>Impl Status (2026-07-03)</t>
         </is>
       </c>
     </row>
@@ -813,7 +885,7 @@
           <t>Display General Information: Order ID/Number, Date Created, Order Status</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -823,19 +895,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Order has order_number (unique), created_at, status — all populated by both built checkout write-paths. Only a net-new GET details endpoint must be built; data primitives exist and are written.</t>
+          <t>CONFIRMED 2026-07-03. order_number/status/created_at on Order, populated by both checkout paths; GET :id detail aggregate is net-new and is the story's core route.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1542 (order_number),1546 (status),1581 (created_at); write-path admin-backend-api/src/admin/cart/services/checkout.service.ts:249; exhibitor-backend-api/src/payments/services/payments.service.ts:186</t>
+          <t>schema order_number:1543/status:1547/created_at:1586; route inventory re-verified on dev@34c6fb4</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -852,7 +920,7 @@
       </c>
       <c r="L2" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -867,9 +935,9 @@
           <t>Order Status taxonomy: Active (Payment Pending), Active (Paid In Full), Cancelled (Full/Partial/No/Never Paid Refund) with automated vs manual transitions per Order Status sheet</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable — sequenced intra-release (24.9)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -877,24 +945,20 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>OrderStatus enum has only pending/partially_paid/completed/failed/refunded/canceled. Active states map to pending+completed (auto, set by webhook), but the four Cancelled refund-substates (full/partial/no/never refund) are not representable; there is no manual status-update endpoint and no refund-aware cancel logic. Displaying the 6-state model and manual-update behavior must be built; the refund substates depend on refund handling that has no code.</t>
+          <t>D1 = option (b): derived status_display, NO enum migration. Active pair from stored enum (pending/partially_paid -&gt; Payment Pending; completed -&gt; Paid In Full); the four Cancelled qualifiers = arithmetic over 24.9's per-installment refund ledger (Never Paid paid=0 / No Refund refunded=0 / Partial 0&lt;r&lt;p / Full r=p). Status Breakdowns tab confirms: stored overall notion is just 'Active'; richness is per-milestone. Installment label map: succeeded-&gt;Paid, scheduled-&gt;Unpaid, failed-&gt;CC Failed, canceled-&gt;Voided, refunded-&gt;Refunded; chargeback trio stays ND per 24.8-l (this sheet is its source). BA note: spec has NO standalone 'Refunded' top-level — refund w/o cancel stays Active; 'failed' maps to Active (Payment Pending).</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:421-430 (OrderStatus enum); paid_in_full_at/paid_amount at schema.prisma:1573-1574</t>
+          <t>OrderStatus enum :421-430; Status Breakdowns tab rows 12-18; sheet fetched in full (6 tabs) 2026-07-03; 24.9 gate D1 (derived refund state)</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Order Status sheet transition rules + refund/void execution path (Order Management refund/void stories)</t>
+          <t>24.9 refund ledger — same release; label map = C13 shared unit</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -910,7 +974,7 @@
       </c>
       <c r="L3" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Partial -&gt; Deliverable-sequenced (D1 option b).</t>
         </is>
       </c>
     </row>
@@ -925,7 +989,7 @@
           <t>Display and (admin) edit Internal Notes</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -935,19 +999,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>RE-VERDICTED 2026-07-03 (was Partial): 24.14 added Order.internal_notes (Text, blank at checkout) with the canonical PATCH /orders/:id/notes edit path + per-field audit. 24.6 only displays the column in its GET details aggregate. Order.notes remains RESERVED (exhibitor checkout idempotency-key store) — never expose it.</t>
+          <t>CONFIRMED 2026-07-03. Column + GET/PATCH :id/notes live via 24.14. Display-only here. Order.notes (:1571) RESERVED — exhibitor idempotency-key store, NEVER expose.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Order.internal_notes shipped by 24.14 (SBE-1138) admin migration 20260702120000_add_order_admin_note_columns; write path src/admin/orders/order-notes.service.ts (merged to dev 2026-07-03, PR#516)</t>
+          <t>Order.internal_notes :1572; orders.controller.ts:94/131; migration 20260702120000; perms :1240/:1248</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -968,7 +1028,7 @@
       </c>
       <c r="L4" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable (24.14 flip re-confirmed).</t>
         </is>
       </c>
     </row>
@@ -983,7 +1043,7 @@
           <t>Display/edit Payment Memo</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -993,19 +1053,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>RE-VERDICTED 2026-07-03 (was Not Deliverable): 24.14 added the brand-new Order.payment_memo (Text) with edit via PATCH /orders/:id/notes + audit. 24.6 only displays it. (Order-level; distinct from 24.8's planned installment-level payment_transactions.payment_memo.)</t>
+          <t>CONFIRMED 2026-07-03. Order-level memo live via 24.14; display-only here. Keep distinct from PT.payment_memo (24.8's installment-level check-#/wire-ref field) — two fields, same name; FE must not conflate (BA note carried on 24.8).</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Order.payment_memo shipped by 24.14 (SBE-1138) admin migration 20260702120000_add_order_admin_note_columns; write path src/admin/orders/order-notes.service.ts (merged to dev 2026-07-03, PR#516)</t>
+          <t>Order.payment_memo :1573 (Text)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1026,7 +1082,7 @@
       </c>
       <c r="L5" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1097,7 @@
           <t>Display Invoice Note / PO #</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -1051,19 +1107,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>RE-VERDICTED 2026-07-03 (was Partial): 24.14 added Order.invoice_note (VarChar(255), copied verbatim from the Cart column; blank at checkout, admin-entered). Display is a direct column read — the cart-only limitation is gone, incl. non-cart orders.</t>
+          <t>CONFIRMED 2026-07-03. Column live via 24.14 (VarChar(255), mirrors Cart def). Display-only.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Order.invoice_note shipped by 24.14 (SBE-1138) admin migration 20260702120000_add_order_admin_note_columns; write path src/admin/orders/order-notes.service.ts (merged to dev 2026-07-03, PR#516)</t>
+          <t>Order.invoice_note :1574</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1084,7 +1136,7 @@
       </c>
       <c r="L6" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1151,7 @@
           <t>Display Additional Terms &amp; Conditions</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -1109,19 +1161,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>RE-VERDICTED 2026-07-03 (was Partial): 24.14 added Order.additional_terms (Text, copied verbatim from the Cart column; blank at checkout, admin-entered). Display is a direct column read — the cart-only limitation is gone.</t>
+          <t>CONFIRMED 2026-07-03. Column live via 24.14 (Text, mirrors Cart def). Display-only.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Order.additional_terms shipped by 24.14 (SBE-1138) admin migration 20260702120000_add_order_admin_note_columns; write path src/admin/orders/order-notes.service.ts (merged to dev 2026-07-03, PR#516)</t>
+          <t>Order.additional_terms :1575</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -1142,7 +1190,7 @@
       </c>
       <c r="L7" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1205,7 @@
           <t>Linked Customer with option to view customer profile and the customer's other orders</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -1167,19 +1215,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Order.company_id FK to Company is always set; a companies controller exists for customer profile lookups, and 'other orders' is a simple Order query by company_id (indexed). Net-new linking/serialization only.</t>
+          <t>CONFIRMED 2026-07-03. company relation + index live; profile = existing company module; 'other orders' = shipped 24.1 list filtered by company_id. Include linkage in response — no other backend.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Order.company relation admin-backend-api/prisma/schema.prisma:1584; @@index([company_id]) schema.prisma:1597; companies controller admin-backend-api/src/admin/company-management/company-management.controller.ts:13</t>
+          <t>company relation :1589; @@index([company_id]) :1602; company-management controller live</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1196,7 +1240,7 @@
       </c>
       <c r="L8" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1255,7 @@
           <t>Billing Information display (Company Name, Billing Address, Email, Phone) with Billing Address editable by admin</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -1221,22 +1265,22 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Order carries the full billing snapshot columns (billing_company_name, billing_address/_2/city/state/country/zip, billing_phone, billing_email). They are written in full by the EXHIBITOR self-service path; the ADMIN checkout writes only company_name + first/last + email and leaves address/phone null, so admin-created product orders need either an upstream snapshot fix or a backfill — but display is immediate and the editable-address requirement is a net-new PATCH buildable on these columns regardless.</t>
+          <t>D2 = option (b): display + net-new PATCH :id billing edit SHIP; admin-checkout write gap (only company/first/last/email written — NO address/phone/city/state/zip keys) REGISTERED to Cart Mgmt team (OQ-1), not fixed here: checkout.service.ts is Suman Paul's actively-evolving Cart Mgmt module (c0e1c46 2026-06-11 .. bb94413 2026-06-29) — record-don't-own. Net effect: admin-created orders show empty address/phone until PATCHed; nothing breaks.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>columns admin-backend-api/prisma/schema.prisma:1553-1563; full write exhibitor-backend-api/src/payments/services/payments.service.ts:205-212; admin checkout writes only company/first/last/email at admin-backend-api/src/admin/cart/services/checkout.service.ts:263-266 (no address/phone)</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
+          <t>billing cols :1554-1564; exhibitor full write payments.service.ts:202-212; admin partial write checkout.service.ts:263-266 (blame = Suman Paul, Cart Mgmt)</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Cart Mgmt team upstream fix (OQ-1) — non-blocking</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -1250,7 +1294,7 @@
       </c>
       <c r="L9" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Partial -&gt; Deliverable (D2 option b, gap registered).</t>
         </is>
       </c>
     </row>
@@ -1265,9 +1309,9 @@
           <t>Email Address with option to add Additional Emails</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1275,22 +1319,22 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>The primary email is backed by Order.billing_email (written on both paths), so display is Deliverable. But there is NO additional-emails collection on Order; Cart's share_email JSON is a one-off cc/bcc snapshot for the share-cart email, not a reusable per-order additional-emails store. Adding additional emails requires a net-new column/table (no upstream dependency, but no primitive exists today).</t>
+          <t>D5 = option (a): net-new Order.additional_emails Json string-array, edited via PATCH :id, DTO email validation. No existing store (grep additional_email/cc_email = 0; Cart.share_email = one-off snapshot). Child table rejected (no per-email metadata requirement anywhere). CC-on-automated-sends = ONE consolidated BA row (OQ-2) naming all four senders (24.6-r, 24.11, 24.15, 24.5); worst case = one-line CC-append per sender, all still unbuilt.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Order.billing_email schema.prisma:1563; share_email is cart-only JSON (admin-backend-api/src/admin/cart/dto/share-cart.dto.ts); grep additional_email/cc_email across schema returns empty</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
+          <t>billing_email :1564; Cart.share_email :2862 (not reusable)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>BA (CC scope only — column unblocked)</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -1304,7 +1348,7 @@
       </c>
       <c r="L10" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Partial -&gt; Deliverable (D5 option a).</t>
         </is>
       </c>
     </row>
@@ -1319,9 +1363,9 @@
           <t>Sales Representative, Order Created By, and Order Type (Sales Person Sale vs Self-Service) display</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1329,19 +1373,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Order has sales_person_id (nullable; set only for salesperson/referral orders). There is NO created_by or sale-source column on Order — note Order.order_type (subscription/ppl_addon/product) is a different taxonomy, not the Sales-Person-Sale vs Self-Service distinction the spec means. Source can be derived from cart.created_by_type for cart-originated orders, but Order itself does not persist creator/source; for non-cart orders it is unknown. Needs derivation logic and likely new persisted fields.</t>
+          <t>D3 = option (a): read-time derivation, NO new columns. Chain: sales_person_id set -&gt; rep name ('Sales Person Sale') -&gt; cart created_by_type=exhibitor -&gt; 'Self-Service' -&gt; created_by_type=admin -&gt; admin creator name -&gt; no cart (subscription/ppl_addon) -&gt; order_type label. Every product order has cart_id by domain design -&gt; 100% coverage. OrderType enum is the BILLING taxonomy, not this notion. Sheet's prefix table (SLF/PPL/...) confirms source = derived classification. Rep name resolved server-side (salesPerson join + shared name-builder, same as 24.1 list).</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Order.sales_person_id schema.prisma:1575; order_type schema.prisma:1545 (different meaning); checkout sets sales_person_id at admin-backend-api/src/admin/cart/services/checkout.service.ts:270; exhibitor referral set at exhibitor-backend-api/src/ppl/services/checkout.service.ts:178</t>
+          <t>sales_person_id :1580; NO created_by/source col on Order (re-verified @34c6fb4); cart.created_by/type cart.service.ts:251-252; OrderType enum :412</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -1358,7 +1398,7 @@
       </c>
       <c r="L11" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Partial -&gt; Deliverable (D3 option a).</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1413,7 @@
           <t>Display Signer First Name, Last Name, and Sign Date</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -1383,19 +1423,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>OrderAgreement stores signer_first_name, signer_last_name, signed_at (immutable, one per order) and is written by the checkout flow. Direct read.</t>
+          <t>CONFIRMED 2026-07-03. OrderAgreement signer_first/last_name + signed_at written at signing; include-in-aggregate.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>OrderAgreement schema.prisma:1607-1623; written at admin-backend-api/src/admin/cart/services/checkout.service.ts:302</t>
+          <t>OrderAgreement :1612-1638 (signer :1615-1616, signed_at :1618); written checkout.service.ts:302</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -1412,7 +1448,7 @@
       </c>
       <c r="L12" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1463,7 @@
           <t>Order Line Items: product name (linked to product details), show name (linked to show details), included items list, Regular Price/Price/Quantity/Total per item</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -1437,19 +1473,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>OrderItem holds description (name snapshot), product_id (FK), show_product_id (FK to per-show offering), quantity, unit_price, custom_unit_price (sales override → Regular vs effective Price), amount, is_default_included (the 'included items' flag). Product/show links resolve via existing modules. Items written by both checkout paths. Net-new serialization only.</t>
+          <t>CONFIRMED 2026-07-03. OrderItem carries description/quantity/unit_price/custom_unit_price/amount/show_product_id/is_default_included + product FK; mirror exhibitor 13.3 rendering (classifyOrderItems + child-amount folding — copy cross-repo, don't import). COUPON CAVEAT: Order.coupon_code (:1549) never populated at checkout — join cart.coupon.code (13.3-proven).</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>OrderItem schema.prisma:1928-1959; items written at admin-backend-api/src/admin/cart/services/checkout.service.ts:277-292 and exhibitor-backend-api/src/cart/helpers/cart.helpers.ts:48-65</t>
+          <t>OrderItem :1943-1974; exhibitor order-details.service.ts:39/:163 (coupon join), order-details.helpers.ts:104</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -1466,7 +1498,7 @@
       </c>
       <c r="L13" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable (coupon-join caveat carried to plan).</t>
         </is>
       </c>
     </row>
@@ -1481,32 +1513,36 @@
           <t>Per line-item Company Contact Name, Email, and Phone</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Implement here</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SBE-1169/1171 (onsite-contact stories)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>OrderItem has no per-item contact fields (no contact columns in schema.prisma:1928-1959); only order-level billing contact exists. A per-line company contact would have to be sourced from order billing or company contact records (not line-item-specific) or modeled new. Order-level contact is available; true per-item contact is not stored.</t>
+          <t>D6: DEFERRED, aligned with 13.3-w (exhibitor twin, Blocked on same stories). Zero contact columns on OrderItem/CartItem anywhere; 'Company Contact' appears exactly ONCE on the whole Confluence page. Best-fit producer OnsiteBoothContact (exact 3-field match; keyed (company_id, show_id); orders are multi-show -&gt; values differ per item's show) gained producer 2026-07-02 (exhibitor module, Sushobhan Manna, SBE-1165 workstream) + edit story SBE-1171 merged 2026-07-03, but SBE-1169 'View Onsite Boot Contact' (Sprint 5, Ritam Mondal) owns display semantics — do not pre-empt. Revisit when SBE-1169 lands: (company_id, show_id) join + billing-contact fallback = small additive read. BA to ratify interpretation (OQ-3).</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>OrderItem fields admin-backend-api/prisma/schema.prisma:1928-1959 (no contact columns); order-level billing at schema.prisma:1553-1563</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
+          <t>OnsiteBoothContact model (@@unique(company_id, show_id)); producer exhibitor src/onsite-booth-contact/* (upsert :121; commits 79757af/bd9d234); no show_id on Order/Cart (multi-show per fee comments)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>SBE-1169 (To Do, Sprint 5, Ritam Mondal) + SBE-1171 (merged 2026-07-03); producer SBE-1165 shipped</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -1520,7 +1556,7 @@
       </c>
       <c r="L14" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Partial -&gt; Deferred (D6; aligned with 13.3-w).</t>
         </is>
       </c>
     </row>
@@ -1535,9 +1571,9 @@
           <t>Sub-items / Add-on products shown under their parent booth/order item via Parent Order Item reference</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1545,22 +1581,22 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>OrderItem.parent_order_item_id (self-relation OrderItemTree) exists and is set ONLY by the exhibitor cart materialization path (materializeCartToOrder maps parent_cart_item_id→parent_order_item_id). The ADMIN checkout createMany and the exhibitor payments.service order path both OMIT it, so admin-created and PPL/addon orders flatten add-ons with no parent linkage. Display works for exhibitor cart-originated orders only; other paths lack the parent reference until their write-paths set it.</t>
+          <t>D2 (same register as 24.6-h): tree render ships (parent_order_item_id/cart_item_type/OrderItemTree live via 13.3-era migration; mirror classifyOrderItems) with GRACEFUL FLAT FALLBACK — admin checkout omits the linkage, so admin-created orders render flat (amounts correct, nothing breaks). Write gap on the combined cart-team register row (OQ-1). Tree self-heals for post-fix orders; historical tree not reconstructable (register asks cart team to decide backfill).</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>parent_order_item_id schema.prisma:1943; set at exhibitor-backend-api/src/cart/helpers/cart.helpers.ts:53; OMITTED by admin createMany admin-backend-api/src/admin/cart/services/checkout.service.ts:277-290 and exhibitor payments.service.ts:217-233</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
+          <t>parent_order_item_id :1958, cart_item_type :1959, OrderItemTree :1968-1969, index :1972; set only by exhibitor cart.helpers.ts:53; admin checkout + exhibitor payments omit it (grep = 0)</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Cart Mgmt team upstream fix (OQ-1) — non-blocking</t>
+        </is>
+      </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
@@ -1574,7 +1610,7 @@
       </c>
       <c r="L15" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Partial -&gt; Deliverable (flat fallback; gap registered).</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1625,7 @@
           <t>Fees: Cleaning Fee and Booth Setup Fee (auto-calculated based on admin configuration)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -1599,19 +1635,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Order.cleaning_fees and Order.setup_fees are frozen snapshot columns computed at checkout from configuration via cart-pricing and written by the admin checkout. Display is a direct read; auto-calc already happens upstream at order creation. (Note: the exhibitor payments path leaves them at default 0, so non-admin orders may show 0 fees — display still works.)</t>
+          <t>CONFIRMED 2026-07-03. Frozen per-show snapshot columns; admin checkout computes+writes, exhibitor path leaves 0 (reverse asymmetry — appended to OQ-1). Auto-calc is upstream; 24.6 displays the snapshot.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Order.setup_fees/cleaning_fees schema.prisma:1577-1578; populated at admin-backend-api/src/admin/cart/services/checkout.service.ts:255-256</t>
+          <t>setup_fees :1582, cleaning_fees :1583; written checkout.service.ts:255-256</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -1628,7 +1660,7 @@
       </c>
       <c r="L16" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1675,7 @@
           <t>Order Totals: Items Subtotal, Fees, Subtotal, Order Total, Balance Payable, Total Payable</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -1653,19 +1685,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Order carries subtotal, setup_fees, cleaning_fees, tax, total, paid_amount; Balance Payable = total - paid_amount (paid_amount bumped by Stripe webhook). All values are frozen/maintained on the order. The spec's 'centralized billing service' does NOT exist; totals are sourced from order columns (+ in-process cart-pricing), which is sufficient for display.</t>
+          <t>CONFIRMED 2026-07-03. subtotal/tax/total/paid_amount + shipped deriveBalanceDue (fixed-2). Net-new = items-subtotal/fees breakdown over OrderItem (C10 residual). DEVIATION NOTE: no 'centralized billing service' exists anywhere — Order's frozen columns + shared helpers ARE the authoritative source. Balance renders from gross paid_amount minus refunds via 24.9 ledger (24.9 D3).</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>schema.prisma:1547-1551,1573 (subtotal/tax/total/paid_amount); fees at 1577-1578; no centralized billing service (cart-pricing.service.ts is in-process)</t>
+          <t>subtotal :1548, tax :1551, total :1552, paid_amount :1578; deriveBalanceDue live (24.1)</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -1686,7 +1714,7 @@
       </c>
       <c r="L17" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable (deviation noted).</t>
         </is>
       </c>
     </row>
@@ -1701,9 +1729,9 @@
           <t>Payment Plan reference linked to the Saved Cart Payment Plan</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable — sequenced intra-release (24.8)</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1711,22 +1739,22 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>CartPaymentPlan + CartPaymentScheduleEntry exist and are keyed to the cart; Order links via cart_id (nullable). For cart-originated orders the plan is reachable; for subscription/ppl_addon orders (cart_id null) there is no plan. The plan is not directly attached to the order, so a cart_id join with null handling must be built.</t>
+          <t>CONFIRMED 2026-07-03. Plan via Order.cart_id join (null-safe: cart_id null for subscription/ppl_addon by design); installment rows consume 24.8's C13 mapper (build order puts 24.8 first). Next-installment piece independent (24.6-q).</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>CartPaymentPlan schema.prisma:2839; CartPaymentScheduleEntry schema.prisma:2854; Order.cart_id (nullable) schema.prisma:1576</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
+          <t>CartPaymentPlan :2911, CartPaymentScheduleEntry :2926; cart_id nullable :1581</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>24.8 C13 mapper — same release, builds first</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
           <t>[C13 cross-reference] Mostly delivered by building 24.8 (A single PaymentTransaction -&gt; installment-row mapper (Invo…). Residual: the detail aggregate embeds the payment-plan reference + next-installment amount/date (24.6-q), derivable from the same PaymentTransaction projection (next = earliest unpaid by due_date). 24.6-p stays Partial (cart_id linkage caveat).</t>
@@ -1744,7 +1772,7 @@
       </c>
       <c r="L18" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Partial -&gt; Deliverable-sequenced (24.8).</t>
         </is>
       </c>
     </row>
@@ -1759,9 +1787,9 @@
           <t>Next Installment Amount and Next Payment Date</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable — sequenced intra-release (24.8)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1769,22 +1797,22 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>PaymentTransaction rows (one per installment) carry amount, due_date, and status (scheduled), written by checkout and processed by the payment-charge cron (query: status='scheduled' AND due_date&lt;=now, orderBy due_date asc). Next installment = earliest scheduled row by due_date. Built write-path and cron both exist.</t>
+          <t>CONFIRMED 2026-07-03. PT rows carry amount/due_date/status/paid timestamps; @@index([status,due_date]) exists for exactly this query; next installment = earliest scheduled by due_date (3-line query, unblockable). Labels per D1 map (scheduled-&gt;Unpaid, canceled-&gt;Voided, ...).</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>PaymentTransaction schema.prisma:2056-2086 (due_date/status, @@index([status, due_date])); cron background-worker-service/src/jobs/payment-charge/payment-charge.service.ts:64-67</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
+          <t>PaymentTransaction :2073-2103 (index :2103); worker payment-charge.service.ts:24</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>24.8 C13 mapper (labels/rows) — same release</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
           <t>[C13 cross-reference] Mostly delivered by building 24.8 (A single PaymentTransaction -&gt; installment-row mapper (Invo…). Residual: the detail aggregate embeds the payment-plan reference + next-installment amount/date (24.6-q), derivable from the same PaymentTransaction projection (next = earliest unpaid by due_date). 24.6-p stays Partial (cart_id linkage caveat).</t>
@@ -1802,7 +1830,7 @@
       </c>
       <c r="L19" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable-sequenced (24.8).</t>
         </is>
       </c>
     </row>
@@ -1817,32 +1845,32 @@
           <t>Send Order Email: select an email template from a dropdown; save order or send email</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Needs clarification (BA)</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Implement here</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>Hold (small; can slot late)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>notification-template module provides template CRUD/listing (dropdown source); the background-worker MailerService.sendFromTemplate resolves a template and dispatches. A net-new order send-email endpoint that selects a template and dispatches is buildable on these primitives. No order-specific send path exists yet, so it is net-new but unblocked.</t>
+          <t>PARKED at gate (user decision). Capability verified buildable: template listing live (SBE-671); dispatch via ADMIN's own MailerService.sendFromTemplate (mailer.service.ts:192 — worker-mailer citation was stale, applies only to 24.15 cron legs); handler drops into 24.5's live order-actions.service.ts pattern. UNIQUENESS SWEPT: no other Confluence story on ANY page has pick-a-template-and-send (E&amp;S epic manages templates only; salesperson 'Save as Template' = cart composition templates, not email, unimplemented); all existing senders fixed-template. OPEN (OQ-4): recipients (spec silent; proposed default [billing_email] + optional override + 400 if none; send by template ID — sidesteps E&amp;S #21), 'Save order' semantics, dropdown scope. Excluded from plan; slots late without re-sequencing.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/notification-template/notification-template.service.ts; background-worker-service/src/notification/mailer.service.ts:88 (sendFromTemplate)</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
+          <t>admin mailer.service.ts:192; order-actions.service.ts:697/:993 (live pattern); notification-template module; uniqueness sweep 2026-07-03 (both Confluence pages + all 5 repos)</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>BA (OQ-4)</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
           <t>[C11 build-once-reuse] Mostly delivered by building 24.5 (MailerService.sendFromTemplate (renders a NotificationTempl…). Residual: send-email dispatches an admin-SELECTED template (dropdown from notification-template list) — distinct selection UI, same mailer.</t>
@@ -1860,7 +1888,7 @@
       </c>
       <c r="L20" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable -&gt; Needs clarification (parked).</t>
         </is>
       </c>
     </row>
@@ -1875,9 +1903,9 @@
           <t>Agreement: view and download the linked agreement</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>Covered elsewhere</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
@@ -1887,20 +1915,24 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>24.5 (SBE-1129) — LIVE on dev</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>OrderAgreement stores the immutable signature/terms, and AgreementDocumentService.generate(cartId, format) builds a downloadable PDF/DOCX. The generator is keyed off cartId (not orderId) and only renders for cart-originated orders; an order-scoped download endpoint (and a path for non-cart orders) must be built on top of OrderAgreement + the existing builder.</t>
+          <t>CONFIRMED 2026-07-03 — upgraded to LIVE: 24.5 (PR#521, merged 2026-07-03) ships GET :id/agreement.pdf|.docx (SIGNED contract). 24.6 residual = zero on download; aggregate includes agreement block (24.6-k fields) + links.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>OrderAgreement schema.prisma:1607; generate(cartId, format) at admin-backend-api/src/admin/cart/services/agreement-document.service.ts:29</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
+          <t>orders.controller.ts:197/:224 on dev@34c6fb4</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>— delivered</t>
+        </is>
+      </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
           <t>[C6 cross-reference] Fully delivered by building 24.5 (GET /api/v1/orders/:id/agreement.pdf and /agreement.docx (r…) — no separate work.</t>
@@ -1918,7 +1950,7 @@
       </c>
       <c r="L21" s="15" t="inlineStr">
         <is>
-          <t>✅ Delivered by 24.5 (merged to dev 2026-07-03) — signed agreement.docx/.pdf routes live (SBE-1129, PR#521)</t>
+          <t>Gate 2026-07-03: Covered by 24.5 — routes live on dev.</t>
         </is>
       </c>
     </row>
@@ -1933,9 +1965,9 @@
           <t>Every order shall have an Assigned Sales Representative, regardless of creation path</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1943,19 +1975,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Order.sales_person_id is nullable and is intentionally left null for admin-created and self-service carts (set only for salesperson/referral orders). There is no guarantee/backfill that every order has an assigned rep. The Cart carries a Deal Owner (created_by) always, but it is not propagated to the Order as a universal assigned rep. Needs a universal-assignment rule and likely a backfill/derivation.</t>
+          <t>D4: the story text supplies the default — self-service orders display 'Self-Service' (D3 chain); no stored field, no house-account user, no backfill, no BA row. sales_person_id stays nullable; 24.6-u PATCH attaches a real rep any time (story explicitly allows reassignment for self-service orders). Rep name resolved server-side (salesPerson join + shared name-builder).</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Order.sales_person_id nullable schema.prisma:1575; admin-backend-api/src/admin/cart/services/checkout.service.ts:267-270 ('Admin-created or self-service carts carry no sales person')</t>
+          <t>sales_person_id :1580 nullable; checkout comment 'Admin-created or self-service carts carry no sales person' (:267-270); schema re-verified @34c6fb4: no new source cols</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -1972,7 +2000,7 @@
       </c>
       <c r="L22" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Partial -&gt; Deliverable (D4: derivation is the default).</t>
         </is>
       </c>
     </row>
@@ -1987,9 +2015,9 @@
           <t>Reassign the Assigned Sales Representative (Deal Owner) via permission-controlled action</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1997,19 +2025,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>The Cart module implements permission-gated Deal Owner reassignment (resolveDealOwnerUpdate / assertAssignableDealOwner + a deal-owners dropdown endpoint), but it writes Cart.created_by (created_by_type=admin), a different field from Order.sales_person_id. There is NO order-level reassignment endpoint; it must be built reusing the cart's assignable-owner pattern but mapping to sales_person_id.</t>
+          <t>CONFIRMED 2026-07-03. Net-new PATCH :id/sales-rep writing Order.sales_person_id (our module), mirroring the live cart deal-owner pattern (validate active Sales-Team/Admin target); dropdown = reuse/mirror GET carts/deal-owners (plan-time choice). Permission key + audit. HubSpot side-effect explicitly NOT attached (OQ-5).</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>cart reassign admin-backend-api/src/admin/cart/services/cart.service.ts:339,418-426 (writes created_by); deal-owners dropdown admin-backend-api/src/admin/cart/cart.controller.ts:572-582</t>
+          <t>cart.service.ts:415-427 (deal-owner helper); cart.controller.ts:612-624 (dropdown)</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -2026,7 +2050,7 @@
       </c>
       <c r="L23" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Partial -&gt; Deliverable.</t>
         </is>
       </c>
     </row>
@@ -2041,34 +2065,30 @@
           <t>Changing the Assigned Sales Rep (Deal Owner) shall automatically update the Deal Owner in HubSpot</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>Needs clarification (BA)</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Implement here</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>HubspotClientService has createContact/updateContact/createCompany/updateCompany/createDeal but NO updateDeal method and NO owner-property update; crucially there is NO order→HubSpot deal linkage (Order has no hubspot_deal_id column — only CompanySubscription and an attendee model carry one) and no code ever creates a deal for an order (createDeal is called only by the nunify attendee webhook). Until an order is linked to a HubSpot deal and an updateDeal/owner capability exists, deal-owner sync cannot run.</t>
+          <t>PARKED at gate (user decision; was Blocked). Three missing layers: NO updateDeal/owner-update on client; NO order-&gt;deal linkage; NO hubspot_deal_id on Order (only CompanySubscription :624 + attendee :2525). NO OWNING EPIC EXISTS: Jira's only CRM epic SBE-1307 = inbound-lead scope (To Do, unassigned); no HubSpot epic on either Confluence page. Inventory (OQ-5): 4.8 post-registration CONTACT sync = the only implemented piece; Onsite Sales deal story unbuilt; Nunify webhook = sole createDeal caller. Sheet's Hubspot tab (pipeline-per-prefix + deal stages) = ready spec input for whoever owns it.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>hubspot client external-api-service/src/modules/hubspot/services/hubspot-client.service.ts:77-200 (createDeal at 173, no updateDeal); only caller external-api-service/src/modules/webhook/services/nunify-webhook.service.ts:254; hubspot_deal_id only on schema.prisma:623 (CompanySubscription) &amp; 2506 (attendee), NOT on Order:1540-1604</t>
+          <t>hubspot-client.service.ts:55-199 (createDeal :173, no updateDeal); nunify-webhook.service.ts:254; exhibitor auth.service.ts:366 (4.8 contact sync live)</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Order→HubSpot deal creation/linkage (hubspot_deal_id on Order) + updateDeal(owner) capability (HubSpot/CRM integration epic)</t>
+          <t>BA (OQ-5: create/route a deal-sync epic)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -2084,7 +2104,7 @@
       </c>
       <c r="L24" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started (Blocked — Order→HubSpot deal creation/linkage (hubspot_deal_id on Order) + updateDeal(owner) capability (HubSpot/CRM integration epic))</t>
+          <t>Gate 2026-07-03: Blocked -&gt; Needs clarification (no owning epic — BA).</t>
         </is>
       </c>
     </row>
@@ -2099,34 +2119,34 @@
           <t>QuickBooks Force Sync: manually sync Invoices, Payments, and Customers to QuickBooks</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C25" s="19" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Implement here</t>
+          <t>Hold</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Epic 65 (QuickBooks)</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>There is ZERO QuickBooks integration code in any repo — grep for quickbooks/intuit across all src returns only 'future module' comments (product income-account placeholders) and dormant schema columns (quickbooks_order_id, quickbooks_sync_status, quickbooks_invoice_id) that nothing writes meaningfully. A full QuickBooks client + sync service must be built before any force-sync action can function.</t>
+          <t>CONFIRMED 2026-07-03: Blocked on epic 65. Zero QB code in all 5 repos ('future module' comments + dormant Order.quickbooks_*/Invoice QB columns written by nothing). Owner exists: epic 65 'Quickbooks Integration/Invoice Creation Process' (Page 2, stories 65.1-65.5, un-ticketed in Jira; missing refund/credit-memo + dispute stories — BA flags from 24.9/24.8 gates). Sheet's QB column cited for that epic (invoices, received payments, credit memos, chargeback journal entries).</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>dormant columns Order.quickbooks_* schema.prisma:1567-1569, Invoice.quickbooks_* schema.prisma:1973-1975; only refs are 'future module' comments admin-backend-api/src/admin/product-management/product-management.service.ts:162-163; no client found</t>
+          <t>dormant cols :1568-1570 + Invoice model; grep quickbooks/intuit = comments only; Page 2 epic 65 (65.1-65.5)</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>QuickBooks integration service (Integrations/QuickBooks epic) — gates this requirement</t>
+          <t>Epic 65 (QuickBooks) — external, un-ticketed</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -2142,7 +2162,7 @@
       </c>
       <c r="L25" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started (Blocked — QuickBooks integration service (Integrations/QuickBooks epic) — gates this requirement)</t>
+          <t>Gate 2026-07-03: Blocked on epic 65 (re-confirmed).</t>
         </is>
       </c>
     </row>
@@ -2157,32 +2177,32 @@
           <t>HubSpot manual sync: manually sync Order to HubSpot</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>Needs clarification (BA)</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Implement here</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>A HubSpot client (create/update contact/company, createDeal) is built, so a manual create-and-sync action can reuse those primitives. But there is no order→deal mapping, no hubspot_deal_id on Order to persist the returned id, no updateDeal for re-sync, and no order-to-HubSpot sync service; the order-field-to-deal mapping and deal-id persistence are net-new and currently missing.</t>
+          <t>D7, PARKED with 24.6-v (same OQ-5 row; v = automatic owner sync, x = manual order sync). createDeal exists but create-once-no-resync = duplicate deals on second click; hubspot_deal_id migration + mapping would pre-empt the unowned epic's design. Nothing built.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>hubspot client external-api-service/src/modules/hubspot/services/hubspot-client.service.ts:77-200; no order sync path; no hubspot_deal_id on Order schema.prisma:1540-1604</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr"/>
+          <t>same as 24.6-v</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>BA (OQ-5)</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
@@ -2196,7 +2216,7 @@
       </c>
       <c r="L26" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Partial -&gt; Needs clarification (with 24.6-v).</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2231,7 @@
           <t>View, edit, refund, void, sync, and reassignment actions are role-based, permission-controlled, and enforced on the backend</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -2221,19 +2241,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>A permission framework exists: RolesGuard reads required permission keys from the Permissions decorator and checks roles_permissions (with a Developer full-access bypass), plus permission-management/role-management modules and a seeder convention for permission keys. New order-action permission keys can be added and enforced on the net-new endpoints.</t>
+          <t>CONFIRMED 2026-07-03. Framework live (roles.guard + roles_permissions + Developer bypass; orders seeder block precedent :1229-1248). Seed keys for SHIPPING actions only (orders.view/update/sales_rep.update/payments.void); refund/cancel keys owned by 24.9/24.10; no keys for parked sync actions.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/auth/guards/roles.guard.ts:8-17 (Developer bypass), :40-86 (permission check); existing per-route @Permissions usage e.g. ppl-order.controller.ts:36,105,130</t>
+          <t>roles.guard.ts :8/:48/:85-86; permission.seeder.ts orders block :1229-1248</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -2254,7 +2270,7 @@
       </c>
       <c r="L27" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -2269,9 +2285,9 @@
           <t>Refund and Void actions available on the order (per Order Status sheet)</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable — refund sequenced (24.9); void 24.6-OWNED</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -2279,24 +2295,20 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>No Stripe refund or void execution path exists: there is no Refund model and no stripe.refunds.create/void anywhere (grep refunds.create/createRefund/stripe.refund returns nothing; the only 'refund' code is a PPL lead-credit refund, unrelated to order payments). stripe_charge_id exists 'for refunds' but nothing consumes it. Surfacing buttons is trivial but the action cannot be delivered until refund/void handling is built; OrderStatus.refunded is set only by the charge.refunded webhook, not by an admin action.</t>
+          <t>SPLIT per sheet's per-row actions (REFUND on paid rows; DELETE+VOID on unpaid/CC-failed rows). Refund half: display flags + wire to 24.9's POST :id/refunds (key orders.refund seeded by 24.9) — zero refund logic here. Void half (D-z, GATE DECISION: 24.6 owns manual per-installment void): POST :id/payments/:transactionId/void, guard status IN (scheduled, failed), sets canceled + next_retry_at:null (24.10 cascade shape — crons never resurrect voided rows), label 'Voided', key orders.payments.void, audited. Distinct from 24.8's scheduled-row delete and 24.10's cancel cascade.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>no Stripe refund code (grep empty across all repos); only PPL lead refund admin-backend-api/src/admin/ppl-service-provider-detail-view/ppl-service-provider-detail-view.service.ts:226; no Refund model in schema; stripe_charge_id schema.prisma:1566</t>
+          <t>Status Breakdowns rows 3-10 (per-milestone actions); worker cron predicates; 24.10 cascade shape (locked 2026-07-03)</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Refund/Void execution path (Stripe refund create + Refund model + admin-initiated cancel/refund logic) — Order Management refund/void stories</t>
+          <t>24.9 (refund flags only) — same release</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2316,7 +2328,7 @@
       </c>
       <c r="L28" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started (Blocked — Refund/Void execution path (Stripe refund create + Refund model + admin-initiated cancel/refund logic) — Order Management refund/void stories)</t>
+          <t>Gate 2026-07-03: Blocked -&gt; Deliverable (refund sequenced; void owned here per gate decision).</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2343,7 @@
           <t>Edit rules: edits blocked for non-editable statuses; signed/completed orders read-only except permitted post-sale actions; field edits enforced on backend</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -2341,19 +2353,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Order.status and OrderAgreement (signed) provide the state needed to gate edits; backend guards can enforce status-based editability on the net-new PATCH endpoints. No status-gating exists for orders yet, but it is buildable on existing fields and the permission framework.</t>
+          <t>CONFIRMED 2026-07-03. Gating state live (status + OrderAgreement presence + guards). Net-new = status-&gt;allowed-actions matrix encoded from the Status Breakdowns action columns (held in full), enforced on 24.6's write routes (billing PATCH blocked post-cancel; post-sale actions per permissions).</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Order.status schema.prisma:1546; OrderAgreement presence schema.prisma:1607; RolesGuard admin-backend-api/src/auth/guards/roles.guard.ts</t>
+          <t>status :1547; OrderAgreement :1612; Status Breakdowns action columns</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -2370,7 +2378,7 @@
       </c>
       <c r="L29" s="15" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2454,281 +2462,235 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>/api/v1/orders/:id</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Full Order Details aggregate: general info, billing snapshot, line items, sub-items, fees, totals + balance, payment plan + next installment, signer/agreement metadata, sales rep/source, customer link.</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>24.6-a, 24.6-b, 24.6-c, 24.6-d, 24.6-e, 24.6-f, 24.6-g, 24.6-h, 24.6-i, 24.6-j, 24.6-k, 24.6-l, 24.6-l2, 24.6-m, 24.6-n, 24.6-o, 24.6-p, 24.6-q</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Opened from the 24.1 list row id (read model); notes/payment-memo/invoice-note/terms display here (columns shipped by 24.14, merged 2026-07-03), their write is on PATCH .../notes.</t>
+      <c r="C2" s="20" t="inlineStr">
+        <is>
+          <t>Full detail aggregate: general, status_display (D1), notes/memo/terms (read-only), billing, additional_emails, customer link, line-item tree (flat fallback) + coupon join, fees, totals + breakdown, plan + installments + next installment, signer/agreement block, sales rep/source (D3).</t>
+        </is>
+      </c>
+      <c r="D2" s="20" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,f,g,h,i,j,k,l,m,n,o,p,q,t</t>
+        </is>
+      </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>Consumes 24.8 C13 mapper, 24.9 ledger, 24.14 columns, 24.5 links</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>PATCH</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>/api/v1/orders/:id</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Admin edit of Billing Address (and order-level fields) with status-based edit rules and backend enforcement.</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>24.6-h, 24.6-aa, 24.6-y</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Notes/invoice-note/terms editing (24.6-c/e/f) was moved off this route to PATCH .../notes (24.14).</t>
-        </is>
-      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>Billing-address + additional_emails edit; status-gated (24.6-aa matrix); audited.</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>h,i,aa,y</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/orders/:id/agreement.pdf</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>View/download the linked order agreement as PDF.</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>24.6-s</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>24.5 — reuses the Quick Actions agreement PDF endpoint; no separate route — reuses 24.5's endpoint.</t>
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>/api/v1/orders/:id/sales-rep</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Reassign rep -&gt; sales_person_id (cart deal-owner pattern); permission-gated; audited. HubSpot side-effect NOT attached (OQ-5).</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>t,u,y</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>Dropdown: reuse/mirror GET carts/deal-owners</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/orders/:id/agreement.docx</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>View/download the linked order agreement as Word/DOCX.</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>24.6-s</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>24.5 — reuses the Quick Actions agreement DOCX endpoint; no separate route — reuses 24.5's endpoint.</t>
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>/api/v1/orders/:id/payments/:transactionId/void</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>24.6-OWNED manual installment void (D-z): guard status IN (scheduled, failed) -&gt; canceled + next_retry_at:null; label 'Voided'.</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>z,y,aa</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>Shape shared w/ 24.10 cascade (same terminal write)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>POST (parked)</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>/api/v1/orders/:id/send-email</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Send an order email using an admin-selected notification template.</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>24.6-r</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>PARKED (OQ-4): template-id send via admin sendFromTemplate; ships only after BA answers recipients/'save order'/dropdown scope.</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>PATCH</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/orders/:id/sales-rep</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Reassign the Assigned Sales Rep / Deal Owner (permission-gated) and trigger the HubSpot Deal Owner update (blocked sub-action).</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>24.6-t, 24.6-u, 24.6-v, 24.6-y</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>GET (live, 24.5)</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>/api/v1/orders/:id/agreement.pdf | .docx</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>LIVE — 24.5's signed-contract routes; 24.6 links only.</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>24.5 (owner)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/orders/:id/hubspot-sync</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Manually sync the order to HubSpot (create contact/company/deal).</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>24.6-x</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>PATCH (live, 24.14)</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>/api/v1/orders/:id/notes</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>LIVE — 24.14's canonical notes write path; 24.6 displays only.</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>c,d,e,f</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>24.14 (owner)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/orders/:id/quickbooks-sync</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Force-sync invoices, payments, and customers to QuickBooks (blocked until a QuickBooks integration exists).</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>24.6-w</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>POST (24.9)</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>/api/v1/orders/:id/refunds</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>24.9's endpoint — 24.6 surfaces per-installment REFUND flags + wiring only.</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>z,b</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>24.9 (owner), 24.11 (email)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/orders/:id/refunds</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Refund action on the order (refund half of 24.6-z).</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>24.6-z</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>24.9 (owner — refund execution), 24.11 (refund email) — no separate route — reuses 24.9's refunds endpoint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/orders/:id/void</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Void action on the order (void half of 24.6-z). BLOCKED — no Stripe void path or Refund model yet.</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>24.6-z</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>PATCH</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/orders/:id/notes</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Edit Internal Notes, Payment Memo, Invoice Note/PO #, and Additional Terms from Order Details.</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>24.6-c, 24.6-d, 24.6-e, 24.6-f</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>24.14 (owner — canonical notes write path, SHIPPED to dev 2026-07-03) — no separate route — reuses 24.14's notes endpoint.</t>
-        </is>
-      </c>
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>(not built)</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>hubspot-sync / quickbooks-sync / order-level void</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>NOT BUILT: hubspot-sync parked (OQ-5); quickbooks-sync Blocked (epic 65); order-level void replaced by per-installment void (D-z).</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>v,w,x</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2741,114 +2703,346 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>Open Question</t>
-        </is>
-      </c>
-      <c r="C1" s="9" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D1" s="9" t="inlineStr">
-        <is>
-          <t>Resolution / Decision</t>
+      <c r="B1" s="21" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="C1" s="21" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D1" s="21" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="E1" s="21" t="inlineStr">
+        <is>
+          <t>Open Question / What is needed</t>
+        </is>
+      </c>
+      <c r="F1" s="21" t="inlineStr">
+        <is>
+          <t>Dependency (blocking story + Jira)</t>
+        </is>
+      </c>
+      <c r="G1" s="21" t="inlineStr">
+        <is>
+          <t>Assignee</t>
+        </is>
+      </c>
+      <c r="H1" s="21" t="inlineStr">
+        <is>
+          <t>Sprint / Jira status</t>
+        </is>
+      </c>
+      <c r="I1" s="21" t="inlineStr">
+        <is>
+          <t>Decision / Current direction</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Spec 'Payment Memo' has no corresponding column anywhere (Order/Cart/Invoice) and is overloaded nowhere — is it a brand-new field or an alias for an existing notes/invoice_note field?</t>
-        </is>
-      </c>
-      <c r="C2" s="15" t="inlineStr">
-        <is>
-          <t>[RESOLVED 2026-07-02, shipped by 24.14 — merged to dev 2026-07-03]</t>
-        </is>
-      </c>
-      <c r="D2" s="15" t="inlineStr">
-        <is>
-          <t>Brand-new Order.payment_memo (Text), distinct from Internal Notes / Invoice Note; order-level, distinct from 24.8's planned installment-level payment_transactions.payment_memo. Edit path = 24.14's PATCH /orders/:id/notes. 24.6-d flipped Not Deliverable → Deliverable (display only).</t>
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>OQ-1</t>
+        </is>
+      </c>
+      <c r="B2" s="20" t="inlineStr">
+        <is>
+          <t>24.6-h, 24.6-m (+n note)</t>
+        </is>
+      </c>
+      <c r="C2" s="20" t="inlineStr">
+        <is>
+          <t>Admin-checkout order snapshot gaps</t>
+        </is>
+      </c>
+      <c r="D2" s="20" t="inlineStr">
+        <is>
+          <t>Deliverable (display ships; upstream gap registered)</t>
+        </is>
+      </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>Admin checkout orders.create (admin src/admin/cart/services/checkout.service.ts, blame c0e1c46/bb94413) omits (1) billing address/phone/city/state/country/zip keys and (2) parent_order_item_id + cart_item_type on items -&gt; admin-created orders show null billing address + flat add-on list. Ask: extend the create call (billing from cart.company; parent map per exhibitor cart.helpers pattern); decide historical backfill. Reverse asymmetry: exhibitor path leaves setup/cleaning fees at 0.</t>
+        </is>
+      </c>
+      <c r="F2" s="20" t="inlineStr">
+        <is>
+          <t>Cart Management epic — un-ticketed; needs a ticket from the cart team</t>
+        </is>
+      </c>
+      <c r="G2" s="20" t="inlineStr">
+        <is>
+          <t>Cart Mgmt team (Suman Paul) via BA/lead</t>
+        </is>
+      </c>
+      <c r="H2" s="20" t="inlineStr">
+        <is>
+          <t>Unticketed as of 2026-07-03</t>
+        </is>
+      </c>
+      <c r="I2" s="20" t="inlineStr">
+        <is>
+          <t>24.6 NOT blocked: nulls/flat render gracefully; billing manually fixable via new PATCH; tree self-heals for post-fix orders. Record-don't-own: we don't edit the cart module.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Should Internal Notes / Invoice Note (PO#) / Additional Terms be snapshotted onto the Order at checkout, or read live from the linked Cart (which leaves subscription/ppl_addon orders, and admin-created orders whose cart may change, without these fields)?</t>
-        </is>
-      </c>
-      <c r="C3" s="15" t="inlineStr">
-        <is>
-          <t>[RESOLVED 2026-07-02, shipped by 24.14 — merged to dev 2026-07-03]</t>
-        </is>
-      </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>Neither snapshot-at-checkout nor cart read-through — the four fields live on Order, created blank at checkout and admin-entered later via PATCH /orders/:id/notes; covers all order types incl. non-cart orders. 24.6-c/e/f flipped Partial → Deliverable (display only).</t>
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>OQ-2</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>24.6-i</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>additional_emails CC scope on automated sends</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>Deliverable (column unblocked)</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>Should Order.additional_emails be CC'd on automated emails? Consumers if yes (one-line CC-append each, all unbuilt): 24.6-r manual send, 24.11 cancel/refund dispatch, 24.15 reminders (carried into its gate), 24.5 resends (note only — shipped). Sheet precedent: refund email offers 'add another email address' (manual, ad-hoc).</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="H3" s="20" t="inlineStr">
+        <is>
+          <t>Open 2026-07-03</t>
+        </is>
+      </c>
+      <c r="I3" s="20" t="inlineStr">
+        <is>
+          <t>Column + PATCH ship regardless; senders default to billing_email until BA answers.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>The 6-state status taxonomy (incl. partial/no/never-refund cancel substates) does not map to the OrderStatus enum — should the enum be extended, or is this a display-only mapping driven by refund records (which do not exist yet)?</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>[OPEN — for team discussion]</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>Current direction (2026-07-01): (pending) — refund cancel substates depend on refund/void records that do not exist yet (24.6-z); resolve once refund/void path + Order Status sheet rules are defined. Gates 24.6-b.</t>
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>OQ-3</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>24.6-l2</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Per-item Company Contact interpretation + revisit</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>Confirm 'Company Contact' on line items = the company's onsite booth contact for the item's show (OnsiteBoothContact, exact 3-field match, per-(company,show) -&gt; differs across show groups). Revisit when SBE-1169 defines display semantics; then a small additive join w/ billing-contact fallback.</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>SBE-1169 View Onsite Boot Contact (+SBE-1171 merged 2026-07-03; producer SBE-1165 shipped 2026-07-02)</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Ritam Mondal (SBE-1169); BA (interpretation)</t>
+        </is>
+      </c>
+      <c r="H4" s="20" t="inlineStr">
+        <is>
+          <t>SBE-1169 To Do, Sprint 5</t>
+        </is>
+      </c>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>Deferred — aligned with 13.3-w; admin must not pre-empt Sprint-5 semantics.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Should the admin checkout path be fixed to snapshot the full billing address/phone and parent_order_item_id (currently only the exhibitor cart path populates these), or will Order Details tolerate null address / flattened add-ons for admin-created orders?</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>[OPEN — for team discussion]</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="inlineStr">
-        <is>
-          <t>Current direction (2026-07-01): (pending) — fixing the admin checkout write-path is cleaner (consistent snapshots), but it is upstream of this read-focused story; team to confirm fix-upstream vs tolerate-nulls. Affects 24.6-h/j/m.</t>
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>OQ-4</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>24.6-r</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>Send Order Email scope</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>Needs clarification</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>(1) Recipients — spec silent; proposed: default [billing_email], optional recipients[] override (billing + additional_emails + ad-hoc), 400 if none. (2) 'Save order or send email' — save WHAT state? (3) Dropdown scope — all active templates or a tagged subset? Uniqueness verified: no other Confluence story anywhere has pick-a-template-and-send; send-by-template-id sidesteps E&amp;S #21.</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>Open 2026-07-03</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>Excluded from plan; small build (handler + DTO into live order-actions pattern) — slots late without re-sequencing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>OQ-5</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>24.6-v, 24.6-x</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>HubSpot deal-sync has NO owning epic</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>Needs clarification</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>Deal-level order sync (auto owner-update v + manual sync x) spec'd only as scattered clauses. Inventory: 4.8 post-registration CONTACT sync implemented (exhibitor auth.service.ts:366 -&gt; external-api client, stores hubspot_contact/company_id); Onsite Sales 'HubSpot Sync' story (Page 2) unbuilt; Nunify attendee webhook = sole createDeal caller; client lacks updateDeal/owner-update; Order lacks hubspot_deal_id. Jira's only CRM epic SBE-1307 = inbound-lead scope. Sheet's Hubspot tab (pipeline-per-order-prefix + stages Closed Won / Closed Lost / Cancelled-No-Refund) = ready spec input. Ask: BA to create/route a deal-sync epic.</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>None exists (that's the issue); nearest: SBE-1307 (different scope, To Do, unassigned)</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>Open 2026-07-03</t>
+        </is>
+      </c>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>24.6 builds nothing HubSpot; 24.6-u ships local reassignment cleanly separable from the future sync side-effect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>OQ-6</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>24.6-b (cross-story)</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Sheet findings routed for BA</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>From Status Breakdowns, in no story's scope: (1) internal cancel notification to departments@theshowproducers.com on every cancel (not in 24.11's locked scope — route or add); (2) refund email send-toggle + extra-recipient ability (extends 24.11's optional-send; conditional one-liner in 24.11's PLAN if ratified); (3) no standalone 'Refunded' overall status — refund w/o cancel stays Active (FE brief). Chargeback trio remains ND per 24.8-l (sheet = source; Jackie Questions tab shows disputes unresolved at accounting level).</t>
+        </is>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="H7" s="20" t="inlineStr">
+        <is>
+          <t>Open 2026-07-03</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>Recorded here (sheet referenced from 24.6); locked sibling docs untouched.</t>
         </is>
       </c>
     </row>
@@ -2863,7 +3057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -2889,70 +3083,87 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>QuickBooks integration service (client + sync of invoices/payments/customers); only dormant quickbooks_* columns and 'future module' comments exist, no code</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>24.6-w (QuickBooks Force Sync)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Integrations / QuickBooks epic</t>
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>QuickBooks integration service — epic 65 'Quickbooks Integration/Invoice Creation Process' (Admin Panel Page 2, stories 65.1-65.5; un-ticketed in Jira; missing refund/credit-memo + dispute stories, BA-flagged at 24.9/24.8 gates; sheet QB column = spec input)</t>
+        </is>
+      </c>
+      <c r="B2" s="20" t="inlineStr">
+        <is>
+          <t>24.6-w</t>
+        </is>
+      </c>
+      <c r="C2" s="20" t="inlineStr">
+        <is>
+          <t>Epic 65 (QuickBooks)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Order→HubSpot deal creation &amp; linkage (hubspot_deal_id on Order) plus an updateDeal/owner capability on the HubSpot client; deals are currently created only for the nunify attendee webhook</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>24.6-v (auto-update Deal Owner in HubSpot) and partly 24.6-x</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>HubSpot / CRM integration epic</t>
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>HubSpot deal-sync epic (DOES NOT EXIST — OQ-5): updateDeal/owner capability + order-&gt;deal linkage + hubspot_deal_id on Order; sheet Hubspot tab = spec input</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>24.6-v, 24.6-x</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>BA to create/route (nearest existing: SBE-1307, inbound-lead scope only)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Refund/Void execution path (Stripe refund create + Refund model + admin-initiated cancel/refund logic); no such code exists</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>24.6-z (refund/void actions) and the refund-based Cancelled substates in 24.6-b</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Order Management refund/void stories</t>
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Onsite-contact display semantics — SBE-1169 (Sprint 5); producer SBE-1165 shipped 2026-07-02; edit SBE-1171 merged 2026-07-03</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>24.6-l2</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Exhibitor Onboarding epic SBE-1075 (Ritam Mondal)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Order Status sheet definition of automated vs manual transitions and per-status allowed actions</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>24.6-b (status taxonomy &amp; behavior)</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Order Management status-definition story</t>
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Admin-checkout snapshot fixes (billing + item tree — OQ-1); non-blocking display-fidelity gap for admin-created orders</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>24.6-h, 24.6-m</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>Cart Management team (Suman Paul)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>In-release (NOT external): 24.9 ledger (b qualifiers, z flags, balance); 24.8 C13 mapper (p/q rows + D1 label map); 24.14 notes columns (c/d/e/f, live); 24.5 agreement routes + order-actions pattern (s live, r's home)</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>24.6-b/p/q/z/c/d/e/f/s</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Same release — build order 24.9-&gt;24.10-&gt;24.11-&gt;24.8-&gt;24.7-&gt;24.6</t>
         </is>
       </c>
     </row>
@@ -2987,182 +3198,182 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
-        <is>
-          <t>Not started — analysis/feasibility stage only. No branch, no SBE ticket, no PR, no Swagger tag. Per-requirement build status is ◻ Not started.</t>
+      <c r="B2" s="20" t="inlineStr">
+        <is>
+          <t>Not started — Step-1 gate complete 2026-07-03 (full 28-item walkthrough with Prantik). Scope locked: 22 Deliverable / 1 Deferred / 3 Needs clarification (BA) / 1 Covered by 24.5 (live) / 1 Blocked (epic 65). Release model: ship-together; builds after 24.8 in the release order.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
-        <is>
-          <t>— (not started)</t>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>SBE ticket</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>SBE-1130 (In Progress, Prantik Saha)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>Commits</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>PR</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>Remaining — all in-scope</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>Everything is remaining: 24.6-a, 24.6-b, 24.6-c, 24.6-d, 24.6-e, 24.6-f, 24.6-g, 24.6-h, 24.6-i, 24.6-j, 24.6-k, 24.6-l, 24.6-l2, 24.6-m, 24.6-n, 24.6-o, 24.6-p, 24.6-q, 24.6-r, 24.6-t, 24.6-u, 24.6-v, 24.6-w, 24.6-x, 24.6-y, 24.6-z, 24.6-aa. (24.6-s is covered elsewhere by 24.5.)</t>
-        </is>
-      </c>
-    </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>Resolved decision — Payment Memo (24.6-d)</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
-        <is>
-          <t>RESOLVED by 24.14 (merged 2026-07-03): brand-new Order.payment_memo, edit via PATCH /orders/:id/notes. 24.6-d flipped to Deliverable (display only).</t>
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Swagger tag</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>Resolved decision — Notes sourcing (24.6-c/e/f)</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>RESOLVED by 24.14 (merged 2026-07-03): columns live on Order, blank at checkout, admin-entered via PATCH /orders/:id/notes. 24.6-c/e/f flipped to Deliverable (display only).</t>
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Build gates</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>Open decision — Status taxonomy (24.6-b)</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>Extend the OrderStatus enum for the 6-state model incl. refund cancel substates, or display-only mapping driven by refund records (which do not exist yet)?</t>
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Live smoke</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>Open decision — Admin-checkout snapshots (24.6-h/j/m)</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Fix admin checkout to snapshot full billing address/phone + parent_order_item_id, or tolerate null address / flattened add-ons for admin-created orders?</t>
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Confirmed build scope</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>GET :id aggregate (incl. derived status_display + rep/source derivation + tree w/ flat fallback + coupon join + plan/installments via C13) · PATCH :id (billing + additional_emails, status-gated) · PATCH :id/sales-rep · POST :id/payments/:transactionId/void (D-z) · Order.additional_emails migration · permission seeds · refund flags wired to 24.9</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>Dependency — 24.5</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="inlineStr">
-        <is>
-          <t>DELIVERED: 24.5's signed agreement PDF/DOCX routes merged to dev 2026-07-03 (SBE-1129, PR#521); no separate route here.</t>
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>Parked pending BA</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>24.6-r send-email (OQ-4) · 24.6-v/x HubSpot (OQ-5)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>Dependency — Integrations / QuickBooks epic</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>QuickBooks integration service (client + sync of invoices/payments/customers) — gates 24.6-w.</t>
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>24.6-l2 onsite contact (SBE-1169/1171 — OQ-3)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>Dependency — HubSpot / CRM integration epic</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>Order→HubSpot deal creation &amp; linkage (hubspot_deal_id on Order) + updateDeal/owner capability — gates 24.6-v and partly 24.6-x.</t>
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>Blocked external</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>24.6-w QuickBooks (epic 65)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Dependency — Order Management refund/void stories</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>Refund/Void execution path (Stripe refund create + Refund model + admin-initiated cancel/refund logic) — gates 24.6-z and refund substates in 24.6-b.</t>
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>External dependencies — see Cross-Epic Dependencies</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>Cart-team snapshot fixes (OQ-1, non-blocking); in-release: 24.9 ledger + 24.8 mapper</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Dependency — Order Management status-definition story</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="inlineStr">
-        <is>
-          <t>Order Status sheet: automated vs manual transitions + per-status allowed actions — gates 24.6-b.</t>
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>Out of API scope</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>FE wiring (navigation, buttons, dropdown UI); HubSpot/QB UI affordances for parked actions</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Out of API scope</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>Front-end wiring (row-to-detail navigation, action buttons). Blocked items (24.6-v/w/z) and 24.6-s are delivered by the owning stories/epics above, not by 24.6.</t>
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>Evidence baseline</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>Verified @admin 0ac2769 (+4 siblings) 2026-07-03; dev moved same day to 34c6fb4 (24.5 PR#521, SBE-1171 PR#520, id-encryption PR#455) — folded in; schema line cites @0ac2769, spot-refresh at plan time.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-management): 24.6 close-out reconfirmation — SBE-1169 DEV DONE (l2 dependency cleared), HubSpot updateDeal now exists (v/x owner-sync still unbuilt)
Post-merge reconfirmation (2026-07-06) against merged dev code + Confluence + Jira:
- 22 Deliverable items re-verified in code (four owned service bodies read in full); no doc drift.
- 24.6-l2: blocker SBE-1169 'View Onsite Boot Contact' now DEV DONE (Release 3, parent SBE-1071) -> dependency cleared; now a buildable native admin read, deferred this release on BA interpretation only (OQ-3).
- 24.6-v/x: HubSpot client updateDeal primitive now exists (subscription-only) -> supersedes 'no updateDeal' note, but order->deal linkage + hubspot_deal_id on Order + SBE-user->hubspot_owner_id owner mapping + owning epic still missing; Needs-clarification (BA) verdict stands.
- 24.6-r (buildable now, BA-only), 24.6-s (delivered by 24.5), 24.6-w (QuickBooks, epic 65 un-ticketed) unchanged.
</commit_message>
<xml_diff>
--- a/order_management/24.6-order-details/24.6 - Order Details.xlsx
+++ b/order_management/24.6-order-details/24.6 - Order Details.xlsx
@@ -1536,7 +1536,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>D6: DEFERRED, aligned with 13.3-w (exhibitor twin, Blocked on same stories). Zero contact columns on OrderItem/CartItem anywhere; 'Company Contact' appears exactly ONCE on the whole Confluence page. Best-fit producer OnsiteBoothContact (exact 3-field match; keyed (company_id, show_id); orders are multi-show -&gt; values differ per item's show) gained producer 2026-07-02 (exhibitor module, Sushobhan Manna, SBE-1165 workstream) + edit story SBE-1171 merged 2026-07-03, but SBE-1169 'View Onsite Boot Contact' (Sprint 5, Ritam Mondal) owns display semantics — do not pre-empt. Revisit when SBE-1169 lands: (company_id, show_id) join + billing-contact fallback = small additive read. BA to ratify interpretation (OQ-3).</t>
+          <t>D6: DEFERRED, aligned with 13.3-w. Zero contact columns on OrderItem/CartItem anywhere; 'Company Contact' appears exactly ONCE on the whole Confluence page. Best-fit producer OnsiteBoothContact (exact 3-field match; keyed (company_id, show_id); orders are multi-show -&gt; values differ per item's show) has producer (exhibitor module, SBE-1165, 2026-07-02) + edit story SBE-1171 (merged 2026-07-03). RECONFIRMED 2026-07-06: SBE-1169 'View Onsite Boot Contact' is now DEV DONE (fixVersion Release 3, parent SBE-1071) — the display-semantics dependency has CLEARED. The (company_id, show_id) join + billing-contact fallback is now a small additive NATIVE ADMIN READ. Stays Deferred (not built this release), parked only on BA interpretation (OQ-3) + 13.3-w parity — no longer blocked on an unbuilt story.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>SBE-1169 (To Do, Sprint 5, Ritam Mondal) + SBE-1171 (merged 2026-07-03); producer SBE-1165 shipped</t>
+          <t>SBE-1169 DEV DONE (Release 3, Ritam Mondal; parent SBE-1071) + SBE-1171 (merged 2026-07-03); producer SBE-1165 shipped [reconfirmed 2026-07-06]</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -2084,12 +2084,12 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>PARKED at gate (user decision; was Blocked). Three missing layers: NO updateDeal/owner-update on client; NO order-&gt;deal linkage; NO hubspot_deal_id on Order (only CompanySubscription :624 + attendee :2525). NO OWNING EPIC EXISTS: Jira's only CRM epic SBE-1307 = inbound-lead scope (To Do, unassigned); no HubSpot epic on either Confluence page. Inventory (OQ-5): 4.8 post-registration CONTACT sync = the only implemented piece; Onsite Sales deal story unbuilt; Nunify webhook = sole createDeal caller. Sheet's Hubspot tab (pipeline-per-prefix + deal stages) = ready spec input for whoever owns it.</t>
+          <t>PARKED at gate (user decision; was Blocked). RECONFIRMED 2026-07-06: the client updateDeal primitive NOW EXISTS (hubspot-client.service.ts:189) — supersedes the earlier 'no updateDeal' note — BUT it is subscription-only (sole caller webhook.service.ts:1019 -&gt; upsertSubscriptionDeal) and the deal-OWNER piece is still absent: (1) NO order-&gt;deal linkage; (2) NO hubspot_deal_id on Order (only CompanySubscription :630 + AttendeeShow :2631); (3) NO owner-id mapping (only hubspot-deals salespersonProperty = affiliate-attribution TEXT, not a hubspot_owner_id / SBE-user-&gt;owner map); (4) NO OWNING EPIC (SBE-1307 = inbound-lead scope, To Do, unassigned). Verdict Needs-clarification (BA) stands.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>hubspot-client.service.ts:55-199 (createDeal :173, no updateDeal); nunify-webhook.service.ts:254; exhibitor auth.service.ts:366 (4.8 contact sync live)</t>
+          <t>hubspot-client.service.ts:173 createDeal / :189 updateDeal (subscription-only via webhook.service.ts:1019); Order has NO hubspot_deal_id (Order block); exhibitor auth.service.ts:366 (4.8 contact sync live) [reconfirmed 2026-07-06]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2196,7 +2196,7 @@
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>D7, PARKED with 24.6-v (same OQ-5 row; v = automatic owner sync, x = manual order sync). createDeal exists but create-once-no-resync = duplicate deals on second click; hubspot_deal_id migration + mapping would pre-empt the unowned epic's design. Nothing built.</t>
+          <t>D7, PARKED with 24.6-v (same OQ-5 row; v = automatic owner sync, x = manual order sync). RECONFIRMED 2026-07-06: client updateDeal now exists (:189) but is subscription-only; create-once-no-resync still risks duplicate deals, and there is still no order-&gt;deal linkage, no hubspot_deal_id on Order, no owner-id mapping, and no owning epic. Nothing built.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2887,12 +2887,12 @@
       </c>
       <c r="E4" s="20" t="inlineStr">
         <is>
-          <t>Confirm 'Company Contact' on line items = the company's onsite booth contact for the item's show (OnsiteBoothContact, exact 3-field match, per-(company,show) -&gt; differs across show groups). Revisit when SBE-1169 defines display semantics; then a small additive join w/ billing-contact fallback.</t>
+          <t>Confirm 'Company Contact' on line items = the company's onsite booth contact for the item's show (OnsiteBoothContact, exact 3-field match, per-(company,show)). RECONFIRMED 2026-07-06: SBE-1169 now DEV DONE — the display-semantics dependency has cleared; the join is now a small additive native admin read w/ billing-contact fallback.</t>
         </is>
       </c>
       <c r="F4" s="20" t="inlineStr">
         <is>
-          <t>SBE-1169 View Onsite Boot Contact (+SBE-1171 merged 2026-07-03; producer SBE-1165 shipped 2026-07-02)</t>
+          <t>SBE-1169 View Onsite Boot Contact — DEV DONE (Release 3) [reconfirmed 2026-07-06] (+SBE-1171 merged 2026-07-03; producer SBE-1165 shipped 2026-07-02)</t>
         </is>
       </c>
       <c r="G4" s="20" t="inlineStr">
@@ -2902,12 +2902,12 @@
       </c>
       <c r="H4" s="20" t="inlineStr">
         <is>
-          <t>SBE-1169 To Do, Sprint 5</t>
+          <t>SBE-1169 DEV DONE, Release 3 (was To Do/Sprint 5) — reconfirmed 2026-07-06</t>
         </is>
       </c>
       <c r="I4" s="20" t="inlineStr">
         <is>
-          <t>Deferred — aligned with 13.3-w; admin must not pre-empt Sprint-5 semantics.</t>
+          <t>Deferred this release — dependency cleared; now a buildable native admin read, parked only on BA interpretation + 13.3-w parity.</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Deal-level order sync (auto owner-update v + manual sync x) spec'd only as scattered clauses. Inventory: 4.8 post-registration CONTACT sync implemented (exhibitor auth.service.ts:366 -&gt; external-api client, stores hubspot_contact/company_id); Onsite Sales 'HubSpot Sync' story (Page 2) unbuilt; Nunify attendee webhook = sole createDeal caller; client lacks updateDeal/owner-update; Order lacks hubspot_deal_id. Jira's only CRM epic SBE-1307 = inbound-lead scope. Sheet's Hubspot tab (pipeline-per-order-prefix + stages Closed Won / Closed Lost / Cancelled-No-Refund) = ready spec input. Ask: BA to create/route a deal-sync epic.</t>
+          <t>Deal-level order sync (auto owner-update v + manual sync x) spec'd only as scattered clauses. Inventory: 4.8 post-registration CONTACT sync implemented (exhibitor auth.service.ts:366); Nunify attendee webhook = sole createDeal caller. RECONFIRMED 2026-07-06: client updateDeal NOW EXISTS (:189) but is subscription-only; STILL MISSING = order-&gt;deal linkage, hubspot_deal_id on Order, SBE-user-&gt;hubspot_owner_id owner mapping (current salespersonProperty is affiliate-attribution text only), and an owning epic. Jira's only CRM epic SBE-1307 = inbound-lead scope. Ask: BA to create/route a deal-sync epic.</t>
         </is>
       </c>
       <c r="F6" s="20" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="H6" s="20" t="inlineStr">
         <is>
-          <t>Open 2026-07-03</t>
+          <t>Open 2026-07-03 (reconfirmed 2026-07-06: updateDeal now exists, owner-sync still unbuilt)</t>
         </is>
       </c>
       <c r="I6" s="20" t="inlineStr">
@@ -3108,7 +3108,7 @@
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
         <is>
-          <t>HubSpot deal-sync epic (DOES NOT EXIST — OQ-5): updateDeal/owner capability + order-&gt;deal linkage + hubspot_deal_id on Order; sheet Hubspot tab = spec input</t>
+          <t>HubSpot deal-sync epic (DOES NOT EXIST — OQ-5). Reconfirmed 2026-07-06: client updateDeal now exists but is subscription-only; still missing = order-&gt;deal linkage + hubspot_deal_id on Order + SBE-user-&gt;hubspot_owner_id owner mapping + an owning epic; sheet Hubspot tab = spec input</t>
         </is>
       </c>
       <c r="B3" s="20" t="inlineStr">
@@ -3125,7 +3125,7 @@
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t>Onsite-contact display semantics — SBE-1169 (Sprint 5); producer SBE-1165 shipped 2026-07-02; edit SBE-1171 merged 2026-07-03</t>
+          <t>Onsite-contact display semantics — SBE-1169 now DEV DONE (Release 3) [reconfirmed 2026-07-06]; producer SBE-1165 shipped 2026-07-02; edit SBE-1171 merged 2026-07-03. Dependency cleared; 24.6-l2 now a buildable native admin read, deferred this release on BA interpretation only</t>
         </is>
       </c>
       <c r="B4" s="20" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>Exhibitor Onboarding epic SBE-1075 (Ritam Mondal)</t>
+          <t>Exhibitor Onboarding (SBE-1071 parent, Ritam Mondal)</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>24.6-l2 onsite contact (SBE-1169/1171 — OQ-3)</t>
+          <t>24.6-l2 onsite contact — dependency SBE-1169 now DEV DONE (reconfirmed 2026-07-06); buildable as a native admin read, parked only on BA interpretation (OQ-3)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-management): 24.6-l2 onsite booth contacts delivered (PR#542)
Flip 24.6-l2 Deferred -> Delivered across the 24.6 story doc (.md/.xlsx),
D6/OQ-3/cross-epic/endpoints reconciled (23 Deliverable / 0 Deferred);
correct the stale billing-contact-fallback note to null-when-absent.
Update OM_PHASE1_RELEASE_PLAN.md (+7 story copies) and the shared-unit
ledger to record the per-show onsite_contacts follow-up.
</commit_message>
<xml_diff>
--- a/order_management/24.6-order-details/24.6 - Order Details.xlsx
+++ b/order_management/24.6-order-details/24.6 - Order Details.xlsx
@@ -642,7 +642,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>SCOPE LOCKED at Step-1 gate 2026-07-03. 22 Deliverable / 1 Deferred / 3 Needs clarification (BA) / 1 Covered elsewhere (24.5, live) / 1 Blocked (epic 65). Ship-together release; builds after 24.8.</t>
+          <t>SCOPE LOCKED at Step-1 gate 2026-07-03. 22 Deliverable / 1 Deferred / 3 Needs clarification (BA) / 1 Covered elsewhere (24.5, live) / 1 Blocked (epic 65). Ship-together release; builds after 24.8. (Post-gate: 24.6-l2 delivered 2026-07-06 as a follow-up → current 23 Deliverable / 0 Deferred.)</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>1 Deferred (l2) · 3 Needs clarification (r, v, x) · 1 Covered by 24.5 (s) · 1 Blocked (w)</t>
+          <t>0 Deferred · 3 Needs clarification (r, v, x) · 1 Covered elsewhere (s→24.5) · 1 Blocked (w→epic 65). 24.6-l2 delivered 2026-07-06 (PR#542).</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10">
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1521,22 +1521,22 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Delivered (follow-up 2026-07-06)</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Implement here</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>SBE-1169/1171 (onsite-contact stories)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>D6: DEFERRED, aligned with 13.3-w. Zero contact columns on OrderItem/CartItem anywhere; 'Company Contact' appears exactly ONCE on the whole Confluence page. Best-fit producer OnsiteBoothContact (exact 3-field match; keyed (company_id, show_id); orders are multi-show -&gt; values differ per item's show) has producer (exhibitor module, SBE-1165, 2026-07-02) + edit story SBE-1171 (merged 2026-07-03). RECONFIRMED 2026-07-06: SBE-1169 'View Onsite Boot Contact' is now DEV DONE (fixVersion Release 3, parent SBE-1071) — the display-semantics dependency has CLEARED. The (company_id, show_id) join + billing-contact fallback is now a small additive NATIVE ADMIN READ. Stays Deferred (not built this release), parked only on BA interpretation (OQ-3) + 13.3-w parity — no longer blocked on an unbuilt story.</t>
+          <t>Delivered 2026-07-06 (PR#542 → dev) once SBE-1169 reached DEV DONE: a per-show onsite_contacts block on GET /orders/:id — one entry per show the order touches (buildOrderShows), each with the company's saved OnsiteBoothContact for that show via one (company_id, show_id) findMany, or contact:null when absent (NO billing fallback; parity with SBE-1169). Native admin read (exhibitor helper not imported). No new route/migration. BA interpretation (OQ-3) ratified by implementation.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="L14" s="20" t="inlineStr">
         <is>
-          <t>Gate 2026-07-03: Partial -&gt; Deferred (D6; aligned with 13.3-w). -&gt; ⏸ DEFERRED (SBE-1169/1171 onsite/booth contact; aligned with 13.3-w) — not built.</t>
+          <t>Delivered 2026-07-06 — commit 8b3f86b, PR#542 → dev; CI + SonarQube gate green.</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="D4" s="22" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Resolved — Delivered</t>
         </is>
       </c>
       <c r="E4" s="20" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="I4" s="20" t="inlineStr">
         <is>
-          <t>Deferred this release — dependency cleared; now a buildable native admin read, parked only on BA interpretation + 13.3-w parity.</t>
+          <t>Resolved — delivered 2026-07-06 (PR#542) in parity with the exhibitor twin 13.3-w; interpretation ratified by implementation (line-item Company Contact = the company's onsite booth contact for that item's show; contact null when absent, no billing fallback).</t>
         </is>
       </c>
     </row>
@@ -3125,12 +3125,12 @@
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t>Onsite-contact display semantics — SBE-1169 now DEV DONE (Release 3) [reconfirmed 2026-07-06]; producer SBE-1165 shipped 2026-07-02; edit SBE-1171 merged 2026-07-03. Dependency cleared; 24.6-l2 now a buildable native admin read, deferred this release on BA interpretation only</t>
+          <t>Onsite-contact display semantics — SBE-1169 DEV DONE (Release 3); producer SBE-1165 shipped 2026-07-02; edit SBE-1171 merged. Dependency CLEARED; 24.6-l2 delivered 2026-07-06 (PR#542) as a native admin per-show onsite_contacts read — no longer an open dependency.</t>
         </is>
       </c>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>24.6-l2</t>
+          <t>24.6-l2 (delivered)</t>
         </is>
       </c>
       <c r="C4" s="20" t="inlineStr">
@@ -3326,12 +3326,12 @@
     <row r="12">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Delivered (follow-up)</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>24.6-l2 onsite contact — dependency SBE-1169 now DEV DONE (reconfirmed 2026-07-06); buildable as a native admin read, parked only on BA interpretation (OQ-3)</t>
+          <t>24.6-l2 onsite booth contacts — shipped 2026-07-06 (branch feature/SBE-1125, commit 8b3f86b, PR#542 → dev) once SBE-1169 reached DEV DONE: per-show onsite_contacts block on GET /orders/:id (join (company_id, show_id); null when a show has none, no billing fallback). CI + SonarQube gate green.</t>
         </is>
       </c>
     </row>

</xml_diff>